<commit_message>
Salon Privé : les 21 couleurs données par l'agence
- couleurs reportées vin par vin (COULEURS_AGENCE, couleur_provenance), pictos à jour
- « effervescent » donne le picto bulles
- liste des vins resserrée : 3 pages ; tableur des prix refait ; tableur des couleurs
  manquantes retiré (plus aucun vin sans couleur)
- QUESTIONS point 28, journal, aperçus

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QqpP8TJ4dopGQHx1iLRkQb
</commit_message>
<xml_diff>
--- a/tableur/prix-salon-prive-2026.xlsx
+++ b/tableur/prix-salon-prive-2026.xlsx
@@ -647,7 +647,11 @@
           <t>AOC Cru Bourgeois Haut-Médoc — Château Balac</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n"/>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Rouge</t>
+        </is>
+      </c>
       <c r="D8" s="12" t="n"/>
       <c r="E8" s="12" t="n"/>
       <c r="F8" s="13" t="n"/>
@@ -808,7 +812,11 @@
           <t>AOP Champagne — Trois Crus Brut</t>
         </is>
       </c>
-      <c r="C15" s="12" t="n"/>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>Blanc effervescent</t>
+        </is>
+      </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
           <t>—</t>
@@ -835,7 +843,11 @@
           <t>AOP Champagne — Terroir Blanc</t>
         </is>
       </c>
-      <c r="C16" s="12" t="n"/>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Blanc effervescent</t>
+        </is>
+      </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
           <t>—</t>
@@ -862,7 +874,11 @@
           <t>AOP Champagne — Terroir Meunier</t>
         </is>
       </c>
-      <c r="C17" s="12" t="n"/>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Blanc effervescent</t>
+        </is>
+      </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
           <t>—</t>
@@ -889,7 +905,11 @@
           <t>AOC Champagne — Brut Nature</t>
         </is>
       </c>
-      <c r="C18" s="12" t="n"/>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Blanc effervescent</t>
+        </is>
+      </c>
       <c r="D18" s="12" t="n"/>
       <c r="E18" s="12" t="n"/>
       <c r="F18" s="13" t="n"/>
@@ -908,7 +928,11 @@
           <t>AOC Champagne — Millésime Expression</t>
         </is>
       </c>
-      <c r="C19" s="12" t="n"/>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Blanc effervescent</t>
+        </is>
+      </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
           <t>2018</t>
@@ -1199,7 +1223,11 @@
           <t>AOC Muscadet Sèvre et Maine — L'envol</t>
         </is>
       </c>
-      <c r="C32" s="12" t="n"/>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>Blanc</t>
+        </is>
+      </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
           <t>2023</t>
@@ -1519,7 +1547,11 @@
           <t>AOC Bourgogne Passe-Tout-Grain</t>
         </is>
       </c>
-      <c r="C44" s="12" t="n"/>
+      <c r="C44" s="12" t="inlineStr">
+        <is>
+          <t>Rouge</t>
+        </is>
+      </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
           <t>2025</t>
@@ -1542,7 +1574,11 @@
           <t>Les Bulles du Puits</t>
         </is>
       </c>
-      <c r="C45" s="12" t="n"/>
+      <c r="C45" s="12" t="inlineStr">
+        <is>
+          <t>Rosé effervescent</t>
+        </is>
+      </c>
       <c r="D45" s="12" t="n"/>
       <c r="E45" s="12" t="n"/>
       <c r="F45" s="13" t="n"/>
@@ -2164,7 +2200,11 @@
           <t>IGP Méditerranée — Premières Fleurs</t>
         </is>
       </c>
-      <c r="C69" s="12" t="n"/>
+      <c r="C69" s="12" t="inlineStr">
+        <is>
+          <t>Blanc</t>
+        </is>
+      </c>
       <c r="D69" s="12" t="inlineStr">
         <is>
           <t>2025</t>
@@ -2187,7 +2227,11 @@
           <t>AOC Muscat BDV — Or des Dentelles</t>
         </is>
       </c>
-      <c r="C70" s="12" t="n"/>
+      <c r="C70" s="12" t="inlineStr">
+        <is>
+          <t>Blanc moelleux</t>
+        </is>
+      </c>
       <c r="D70" s="12" t="inlineStr">
         <is>
           <t>2023</t>
@@ -2210,7 +2254,11 @@
           <t>AOC Muscat BDV — Or des Dentelles</t>
         </is>
       </c>
-      <c r="C71" s="12" t="n"/>
+      <c r="C71" s="12" t="inlineStr">
+        <is>
+          <t>Blanc moelleux</t>
+        </is>
+      </c>
       <c r="D71" s="12" t="inlineStr">
         <is>
           <t>2022</t>
@@ -2992,7 +3040,11 @@
           <t>La Grange Jaumain – Grolleau Noir</t>
         </is>
       </c>
-      <c r="C101" s="12" t="n"/>
+      <c r="C101" s="12" t="inlineStr">
+        <is>
+          <t>Rouge</t>
+        </is>
+      </c>
       <c r="D101" s="12" t="inlineStr">
         <is>
           <t>2024</t>
@@ -3325,7 +3377,11 @@
           <t>AOC Bugey — Mas de Lusanne Mondeuse</t>
         </is>
       </c>
-      <c r="C116" s="12" t="n"/>
+      <c r="C116" s="12" t="inlineStr">
+        <is>
+          <t>Rouge</t>
+        </is>
+      </c>
       <c r="D116" s="12" t="inlineStr">
         <is>
           <t>2023</t>
@@ -3348,7 +3404,11 @@
           <t>AOC Bugey — Mas de Lusanne Pinot Noir</t>
         </is>
       </c>
-      <c r="C117" s="12" t="n"/>
+      <c r="C117" s="12" t="inlineStr">
+        <is>
+          <t>Rouge</t>
+        </is>
+      </c>
       <c r="D117" s="12" t="inlineStr">
         <is>
           <t>2023</t>
@@ -3425,7 +3485,11 @@
           <t>AOC Bugey — Mas de Lusanne Gamay</t>
         </is>
       </c>
-      <c r="C120" s="12" t="n"/>
+      <c r="C120" s="12" t="inlineStr">
+        <is>
+          <t>Rouge</t>
+        </is>
+      </c>
       <c r="D120" s="12" t="n"/>
       <c r="E120" s="12" t="n"/>
       <c r="F120" s="13" t="n"/>
@@ -3444,7 +3508,11 @@
           <t>AOC Bugey — Mas de Lusanne Chardonnay</t>
         </is>
       </c>
-      <c r="C121" s="12" t="n"/>
+      <c r="C121" s="12" t="inlineStr">
+        <is>
+          <t>Blanc</t>
+        </is>
+      </c>
       <c r="D121" s="12" t="inlineStr">
         <is>
           <t>2020</t>
@@ -3663,7 +3731,11 @@
           <t>AOC Saint-Chinian — Juliette</t>
         </is>
       </c>
-      <c r="C130" s="12" t="n"/>
+      <c r="C130" s="12" t="inlineStr">
+        <is>
+          <t>Blanc</t>
+        </is>
+      </c>
       <c r="D130" s="12" t="inlineStr">
         <is>
           <t>2025</t>
@@ -4504,7 +4576,11 @@
           <t>AOC Pouilly-Fumé — Vignes de Tréleau</t>
         </is>
       </c>
-      <c r="C165" s="12" t="n"/>
+      <c r="C165" s="12" t="inlineStr">
+        <is>
+          <t>Blanc</t>
+        </is>
+      </c>
       <c r="D165" s="12" t="inlineStr">
         <is>
           <t>2023</t>
@@ -6126,7 +6202,11 @@
           <t>AOC Fronsac — Château Lafargue</t>
         </is>
       </c>
-      <c r="C231" s="12" t="n"/>
+      <c r="C231" s="12" t="inlineStr">
+        <is>
+          <t>Rouge</t>
+        </is>
+      </c>
       <c r="D231" s="12" t="inlineStr">
         <is>
           <t>2020</t>
@@ -6353,7 +6433,11 @@
           <t>IGP Val de Loire — L'Eberluant – Chardonnay</t>
         </is>
       </c>
-      <c r="C240" s="12" t="n"/>
+      <c r="C240" s="12" t="inlineStr">
+        <is>
+          <t>Blanc pétillant</t>
+        </is>
+      </c>
       <c r="D240" s="12" t="inlineStr">
         <is>
           <t>2025</t>

</xml_diff>